<commit_message>
Drop contingency, add 4 Genshin PCs, end day at 18:00
Move reserve into four gaming PCs for the Genshin zone, trim event
production lines to keep 900k, and compress the schedule to close at 18:00.

Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -115,7 +115,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -507,7 +506,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Смета зоны Mobile Legends + Genshin Impact · Киберсуббота · 6 февраля 2027</t>
+          <t>Смета зоны Mobile Legends + Genshin Impact · Киберсуббота · 6 февраля 2027 · до 18:00</t>
         </is>
       </c>
     </row>
@@ -559,59 +558,59 @@
           <t>1. Аренда локаций</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Аренда площадки</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>День мероприятия</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>сутки</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="6" t="n">
+      <c r="E4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>348000</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>348000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Итого: 1. Аренда локаций</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="8" t="n">
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="7" t="n">
         <v>348000</v>
       </c>
     </row>
@@ -621,91 +620,91 @@
           <t>2. Техническое обслуживание зон</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Администратор зоны</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Операционное решение административных вопросов на площадке</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6" t="n">
+      <c r="F7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>7800</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="5" t="n">
         <v>31200</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Технический администратор</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Техническое обеспечение: звук, экран, интернет, коммутация</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="E8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>14400</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="5" t="n">
         <v>14400</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Итого: 2. Техническое обслуживание зон</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="8" t="n">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="7" t="n">
         <v>45600</v>
       </c>
     </row>
@@ -715,187 +714,187 @@
           <t>3. Медиа / трансляция</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Режиссёр трансляции</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Управление эфиром, переключение камер и графики</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="6" t="n">
+      <c r="E11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="5" t="n">
         <v>25000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Обсервер</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Внутриигровая режиссура</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6" t="n">
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>20000</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Инженер по звуку</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Звук на площадке и в трансляции</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="6" t="n">
+      <c r="E13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="5" t="n">
         <v>18000</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="5" t="n">
         <v>18000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Инженер трансляции</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Маршрутизация сигнала, стабильность эфира</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="6" t="n">
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="5" t="n">
         <v>25000</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Режиссёр по графике</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Вывод графики в видеопоток</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="6" t="n">
+      <c r="E15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="5" t="n">
         <v>20000</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Итого: 3. Медиа / трансляция</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="8" t="n">
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="7" t="n">
         <v>108000</v>
       </c>
     </row>
@@ -905,610 +904,614 @@
           <t>4. Оборудование</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Студийный свет</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Комплект студийного света</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>комплект</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="6" t="n">
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="5" t="n">
         <v>26000</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="5" t="n">
         <v>26000</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Игровой компьютер</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Зона Genshin Impact, мини-игры; смена до 12 ч</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>10440</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>41760</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Телевизор 65″</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Зона Genshin Impact и показ на зоне; смена до 12 ч</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E20" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="6" t="n">
+      <c r="F20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H20" s="5" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Итого: 4. Оборудование</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="8" t="n">
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="7" t="n">
+        <v>73760</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>5. Менеджмент</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Менеджмент мероприятия</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Координация зоны и программы</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="6" t="n">
+      <c r="E23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="5" t="n">
         <v>80000</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H23" s="5" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Итого: 5. Менеджмент</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="8" t="n">
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="7" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>6. Организация ивента</t>
         </is>
       </c>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Косплееры Mobile Legends (2 чел.)</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>45000</v>
-      </c>
-      <c r="H25" s="6" t="n">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="E26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Косплеерша Genshin Impact (1 чел.)</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="6" t="n">
+      <c r="E27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="H26" s="6" t="n">
+      <c r="H27" s="5" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="n">
+    <row r="28">
+      <c r="A28" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Фотозона Mobile Legends 3×2 м</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Каркас, печать, монтаж</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="6" t="n">
+      <c r="E28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="5" t="n">
         <v>15000</v>
       </c>
-      <c r="H27" s="6" t="n">
+      <c r="H28" s="5" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="n">
+    <row r="29">
+      <c r="A29" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Декор зоны Genshin Impact</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Панели, ткань, фонари, фотофон</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="6" t="n">
+      <c r="E29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5" t="n">
         <v>30000</v>
       </c>
-      <c r="H28" s="6" t="n">
+      <c r="H29" s="5" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="n">
+    <row r="30">
+      <c r="A30" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Декор под Китайский Новый год</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Зона Mobile Legends и проходы</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E29" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="H29" s="6" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="E30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>21590</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>21590</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Ведущий</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="H30" s="6" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="E31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Алмазы Mobile Legends 15 000 шт.</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Призы</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="6" t="n">
+      <c r="E32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="5" t="n">
         <v>24150</v>
       </c>
-      <c r="H31" s="6" t="n">
+      <c r="H32" s="5" t="n">
         <v>24150</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="n">
+    <row r="33">
+      <c r="A33" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Денежный приз турнира 5×5</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="H32" s="6" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="E33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Бинго и расходники</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E33" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="6" t="n">
+      <c r="E34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="5" t="n">
         <v>6000</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H34" s="5" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="n">
+    <row r="35">
+      <c r="A35" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Покупки в Genshin Impact для зоны</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Валюта и оформление</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E34" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="6" t="n">
+      <c r="E35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H35" s="5" t="n">
         <v>5000</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="n">
+    <row r="36">
+      <c r="A36" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Аренда 14 смартфонов</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>2 суток, с резервом</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E35" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="6" t="n">
+      <c r="E36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="5" t="n">
         <v>15900</v>
       </c>
-      <c r="H35" s="6" t="n">
+      <c r="H36" s="5" t="n">
         <v>15900</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="n">
+    <row r="37">
+      <c r="A37" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Медийный гость</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr"/>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>проект</t>
         </is>
       </c>
-      <c r="E36" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="H36" s="6" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Запас на непредвиденное</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>20350</v>
-      </c>
-      <c r="H37" s="6" t="n">
-        <v>20350</v>
+      <c r="E37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Итого: 6. Организация ивента</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="8" t="n">
-        <v>286400</v>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="7" t="n">
+        <v>244640</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="9" t="n"/>
-      <c r="F39" s="9" t="n"/>
-      <c r="G39" s="9" t="n"/>
-      <c r="H39" s="10" t="n">
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+      <c r="H39" s="9" t="n">
         <v>900000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A23:G23"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A5:G5"/>

</xml_diff>

<commit_message>
Split 348k venue fee into venue service lines in estimate
Replace the single arena rental row with space setup, tech, infra and
day support services totaling 348000 while keeping the 900k Excel smeta.

Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -80,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -102,11 +102,55 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -115,6 +159,8 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -490,11 +536,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -555,967 +601,1095 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. Аренда локаций</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
+          <t>1. Обеспечение площадки</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Аренда площадки</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>День мероприятия</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>сутки</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="5" t="n">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Организация пространства зоны</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Выделение и оформление зоны под программу дня</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>90000</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Подготовка и сетап площадки</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Монтаж зоны до открытия, подготовка рабочих мест</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>55000</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Техническое обеспечение площадки</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Базовый свет, звук и видео инфраструктуры арены</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Инфраструктура и коммутация</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Интернет, экраны арены, коммутация сигналов</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Сопровождение площадки в день мероприятия</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Работа площадки до 18:00</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>58000</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Итого: 1. Обеспечение площадки</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="9" t="n">
         <v>348000</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>348000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Итого: 1. Аренда локаций</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="7" t="n">
-        <v>348000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2. Техническое обслуживание зон</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Администратор зоны</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Операционное решение административных вопросов на площадке</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>чел.</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>31200</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Технический администратор</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Техническое обеспечение: звук, экран, интернет, коммутация</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>чел.</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>14400</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>14400</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Итого: 2. Техническое обслуживание зон</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="7" t="n">
-        <v>45600</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>2. Техническое обслуживание зон</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Администратор зоны</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Операционное решение административных вопросов на площадке</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>7800</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>31200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Технический администратор</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Техническое обеспечение: звук, экран, интернет, коммутация</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>14400</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>14400</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Итого: 2. Техническое обслуживание зон</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="9" t="n">
+        <v>45600</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>3. Медиа / трансляция</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Режиссёр трансляции</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Управление эфиром, переключение камер и графики</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5" t="n">
+      <c r="E15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H15" s="7" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Обсервер</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Внутриигровая режиссура</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="5" t="n">
+      <c r="E16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H16" s="7" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Инженер по звуку</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Звук на площадке и в трансляции</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="5" t="n">
+      <c r="E17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>18000</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H17" s="7" t="n">
         <v>18000</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Инженер трансляции</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Маршрутизация сигнала, стабильность эфира</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="5" t="n">
+      <c r="E18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H18" s="7" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+    <row r="19">
+      <c r="A19" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Режиссёр по графике</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Вывод графики в видеопоток</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="5" t="n">
+      <c r="E19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H19" s="7" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Итого: 3. Медиа / трансляция</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="7" t="n">
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="9" t="n">
         <v>108000</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>4. Оборудование</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Студийный свет</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Комплект студийного света</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>комплект</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="5" t="n">
+      <c r="E22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="7" t="n">
         <v>26000</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H22" s="7" t="n">
         <v>26000</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
+    <row r="23">
+      <c r="A23" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Игровой компьютер</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Зона Genshin Impact, мини-игры; смена до 12 ч</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E23" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="5" t="n">
+      <c r="F23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="7" t="n">
         <v>10440</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="H23" s="7" t="n">
         <v>41760</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+    <row r="24">
+      <c r="A24" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Телевизор 65″</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Зона Genshin Impact и показ на зоне; смена до 12 ч</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E24" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="5" t="n">
+      <c r="F24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H24" s="7" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Итого: 4. Оборудование</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="7" t="n">
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="9" t="n">
         <v>73760</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>5. Менеджмент</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Менеджмент мероприятия</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Координация зоны и программы</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="5" t="n">
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H27" s="7" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Итого: 5. Менеджмент</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="7" t="n">
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="9" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>6. Организация ивента</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Косплееры Mobile Legends (2 чел.)</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="5" t="n">
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="7" t="n">
         <v>40000</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="H30" s="7" t="n">
         <v>40000</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
+    <row r="31">
+      <c r="A31" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Косплеерша Genshin Impact (1 чел.)</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="5" t="n">
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H31" s="7" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+    <row r="32">
+      <c r="A32" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Фотозона Mobile Legends 3×2 м</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Каркас, печать, монтаж</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="5" t="n">
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H32" s="7" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
+    <row r="33">
+      <c r="A33" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Декор зоны Genshin Impact</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Панели, ткань, фонари, фотофон</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="5" t="n">
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="H29" s="5" t="n">
+      <c r="H33" s="7" t="n">
         <v>30000</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+    <row r="34">
+      <c r="A34" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Декор под Китайский Новый год</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Зона Mobile Legends и проходы</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="5" t="n">
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="7" t="n">
         <v>21590</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H34" s="7" t="n">
         <v>21590</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
+    <row r="35">
+      <c r="A35" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Ведущий</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="5" t="n">
+      <c r="C35" s="6" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="7" t="n">
         <v>22000</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H35" s="7" t="n">
         <v>22000</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+    <row r="36">
+      <c r="A36" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Алмазы Mobile Legends 15 000 шт.</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Призы</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="5" t="n">
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="7" t="n">
         <v>24150</v>
       </c>
-      <c r="H32" s="5" t="n">
+      <c r="H36" s="7" t="n">
         <v>24150</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
+    <row r="37">
+      <c r="A37" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Денежный приз турнира 5×5</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="5" t="n">
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H37" s="7" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+    <row r="38">
+      <c r="A38" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Бинго и расходники</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="5" t="n">
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="7" t="n">
         <v>6000</v>
       </c>
-      <c r="H34" s="5" t="n">
+      <c r="H38" s="7" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
+    <row r="39">
+      <c r="A39" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Покупки в Genshin Impact для зоны</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Валюта и оформление</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="5" t="n">
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H39" s="7" t="n">
         <v>5000</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Аренда 14 смартфонов</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>2 суток, с резервом</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="5" t="n">
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="7" t="n">
         <v>15900</v>
       </c>
-      <c r="H36" s="5" t="n">
+      <c r="H40" s="7" t="n">
         <v>15900</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Медийный гость</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="5" t="n">
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="H37" s="5" t="n">
+      <c r="H41" s="7" t="n">
         <v>20000</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Итого: 6. Организация ивента</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="7" t="n">
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="9" t="n">
         <v>244640</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="B39" s="8" t="n"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="8" t="n"/>
-      <c r="G39" s="8" t="n"/>
-      <c r="H39" s="9" t="n">
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="4" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="11" t="n">
         <v>900000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Recalculate estimate so 5% VAT lands on 900k total
Store line items as net amounts, add VAT 5% summary rows, and keep the
gross project total at 900000 RUB in the Excel smeta and brief site.

Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -29,7 +29,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -52,7 +52,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,10 +155,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -169,8 +174,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -549,10 +556,10 @@
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Смета зоны Mobile Legends + Genshin Impact · Киберсуббота · 6 февраля 2027 · до 18:00</t>
+          <t>Смета зоны Mobile Legends + Genshin Impact · Киберсуббота · 6 февраля 2027 · до 18:00 · цены без НДС</t>
         </is>
       </c>
     </row>
@@ -638,10 +645,10 @@
         <v>1</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>90000</v>
+        <v>85714</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>90000</v>
+        <v>85714</v>
       </c>
     </row>
     <row r="5">
@@ -670,10 +677,10 @@
         <v>1</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>55000</v>
+        <v>52381</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>55000</v>
+        <v>52381</v>
       </c>
     </row>
     <row r="6">
@@ -702,10 +709,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>80000</v>
+        <v>76190</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>80000</v>
+        <v>76190</v>
       </c>
     </row>
     <row r="7">
@@ -734,10 +741,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>65000</v>
+        <v>61905</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>65000</v>
+        <v>61905</v>
       </c>
     </row>
     <row r="8">
@@ -766,10 +773,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>58000</v>
+        <v>55238</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>58000</v>
+        <v>55238</v>
       </c>
     </row>
     <row r="9">
@@ -785,7 +792,7 @@
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="9" t="n">
-        <v>348000</v>
+        <v>331428</v>
       </c>
     </row>
     <row r="10">
@@ -828,10 +835,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>7800</v>
+        <v>7428.5</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>31200</v>
+        <v>29714</v>
       </c>
     </row>
     <row r="12">
@@ -860,10 +867,10 @@
         <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>14400</v>
+        <v>13714</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>14400</v>
+        <v>13714</v>
       </c>
     </row>
     <row r="13">
@@ -879,7 +886,7 @@
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="9" t="n">
-        <v>45600</v>
+        <v>43428</v>
       </c>
     </row>
     <row r="14">
@@ -922,10 +929,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
     </row>
     <row r="16">
@@ -954,10 +961,10 @@
         <v>1</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
     </row>
     <row r="17">
@@ -986,10 +993,10 @@
         <v>1</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>18000</v>
+        <v>17143</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>18000</v>
+        <v>17143</v>
       </c>
     </row>
     <row r="18">
@@ -1018,10 +1025,10 @@
         <v>1</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
     </row>
     <row r="19">
@@ -1050,10 +1057,10 @@
         <v>1</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
     </row>
     <row r="20">
@@ -1069,7 +1076,7 @@
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="9" t="n">
-        <v>108000</v>
+        <v>102859</v>
       </c>
     </row>
     <row r="21">
@@ -1112,10 +1119,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>26000</v>
+        <v>24762</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>26000</v>
+        <v>24762</v>
       </c>
     </row>
     <row r="23">
@@ -1144,10 +1151,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>10440</v>
+        <v>9942.75</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>41760</v>
+        <v>39771</v>
       </c>
     </row>
     <row r="24">
@@ -1176,10 +1183,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>3000</v>
+        <v>2857</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>6000</v>
+        <v>5714</v>
       </c>
     </row>
     <row r="25">
@@ -1195,7 +1202,7 @@
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="5" t="n"/>
       <c r="H25" s="9" t="n">
-        <v>73760</v>
+        <v>70247</v>
       </c>
     </row>
     <row r="26">
@@ -1238,10 +1245,10 @@
         <v>1</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>80000</v>
+        <v>76190</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>80000</v>
+        <v>76190</v>
       </c>
     </row>
     <row r="28">
@@ -1257,7 +1264,7 @@
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="9" t="n">
-        <v>80000</v>
+        <v>76190</v>
       </c>
     </row>
     <row r="29">
@@ -1300,10 +1307,10 @@
         <v>1</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>40000</v>
+        <v>38095</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>40000</v>
+        <v>38095</v>
       </c>
     </row>
     <row r="31">
@@ -1332,10 +1339,10 @@
         <v>1</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>25000</v>
+        <v>23810</v>
       </c>
     </row>
     <row r="32">
@@ -1364,10 +1371,10 @@
         <v>1</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>15000</v>
+        <v>14286</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>15000</v>
+        <v>14286</v>
       </c>
     </row>
     <row r="33">
@@ -1396,10 +1403,10 @@
         <v>1</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>30000</v>
+        <v>28571</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>30000</v>
+        <v>28571</v>
       </c>
     </row>
     <row r="34">
@@ -1428,10 +1435,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>21590</v>
+        <v>20562</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>21590</v>
+        <v>20562</v>
       </c>
     </row>
     <row r="35">
@@ -1456,10 +1463,10 @@
         <v>1</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>22000</v>
+        <v>20952</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>22000</v>
+        <v>20952</v>
       </c>
     </row>
     <row r="36">
@@ -1488,10 +1495,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>24150</v>
+        <v>23000</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>24150</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="37">
@@ -1516,10 +1523,10 @@
         <v>1</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
     </row>
     <row r="38">
@@ -1544,10 +1551,10 @@
         <v>1</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>6000</v>
+        <v>5714</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>6000</v>
+        <v>5714</v>
       </c>
     </row>
     <row r="39">
@@ -1576,10 +1583,10 @@
         <v>1</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>5000</v>
+        <v>4762</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>5000</v>
+        <v>4762</v>
       </c>
     </row>
     <row r="40">
@@ -1608,10 +1615,10 @@
         <v>1</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>15900</v>
+        <v>15143</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>15900</v>
+        <v>15143</v>
       </c>
     </row>
     <row r="41">
@@ -1636,10 +1643,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>20000</v>
+        <v>19048</v>
       </c>
     </row>
     <row r="42">
@@ -1655,13 +1662,13 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="5" t="n"/>
       <c r="H42" s="9" t="n">
-        <v>244640</v>
+        <v>232991</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Итого без НДС</t>
         </is>
       </c>
       <c r="B43" s="4" t="n"/>
@@ -1670,18 +1677,52 @@
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="5" t="n"/>
-      <c r="H43" s="11" t="n">
+      <c r="H43" s="9" t="n">
+        <v>857143</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>НДС 5%</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="11" t="n">
+        <v>42857</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>ИТОГО с НДС</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="13" t="n">
         <v>900000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A45:G45"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A20:G20"/>

</xml_diff>

<commit_message>
Refresh Excel smeta with round numbers and 348k venue
Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -169,15 +169,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -645,10 +645,10 @@
         <v>1</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>85714</v>
+        <v>100000</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>85714</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="5">
@@ -677,10 +677,10 @@
         <v>1</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>52381</v>
+        <v>60000</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>52381</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="6">
@@ -709,10 +709,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>76190</v>
+        <v>80000</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>76190</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="7">
@@ -741,10 +741,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>61905</v>
+        <v>60000</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>61905</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="8">
@@ -773,10 +773,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>55238</v>
+        <v>48000</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>55238</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="9">
@@ -792,7 +792,7 @@
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="9" t="n">
-        <v>331428</v>
+        <v>348000</v>
       </c>
     </row>
     <row r="10">
@@ -835,10 +835,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>7428.5</v>
+        <v>7000</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>29714</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="12">
@@ -867,10 +867,10 @@
         <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>13714</v>
+        <v>12000</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>13714</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="13">
@@ -886,7 +886,7 @@
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="9" t="n">
-        <v>43428</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="14">
@@ -929,10 +929,10 @@
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>23810</v>
+        <v>22000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>23810</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="16">
@@ -961,10 +961,10 @@
         <v>1</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>19048</v>
+        <v>18000</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>19048</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="17">
@@ -993,10 +993,10 @@
         <v>1</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>17143</v>
+        <v>15000</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>17143</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="18">
@@ -1025,10 +1025,10 @@
         <v>1</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>23810</v>
+        <v>22000</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>23810</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="19">
@@ -1057,10 +1057,10 @@
         <v>1</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>19048</v>
+        <v>18000</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>19048</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="20">
@@ -1076,7 +1076,7 @@
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="9" t="n">
-        <v>102859</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="21">
@@ -1119,10 +1119,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>24762</v>
+        <v>25000</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>24762</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="23">
@@ -1151,10 +1151,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>9942.75</v>
+        <v>9000</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>39771</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="24">
@@ -1183,10 +1183,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2857</v>
+        <v>3000</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>5714</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="25">
@@ -1202,7 +1202,7 @@
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="5" t="n"/>
       <c r="H25" s="9" t="n">
-        <v>70247</v>
+        <v>67000</v>
       </c>
     </row>
     <row r="26">
@@ -1245,10 +1245,10 @@
         <v>1</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>76190</v>
+        <v>70000</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>76190</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="28">
@@ -1264,7 +1264,7 @@
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="9" t="n">
-        <v>76190</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="29">
@@ -1307,10 +1307,10 @@
         <v>1</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>38095</v>
+        <v>40000</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>38095</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="31">
@@ -1339,10 +1339,10 @@
         <v>1</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>23810</v>
+        <v>25000</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>23810</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="32">
@@ -1371,10 +1371,10 @@
         <v>1</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>14286</v>
+        <v>15000</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>14286</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="33">
@@ -1403,10 +1403,10 @@
         <v>1</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>28571</v>
+        <v>30000</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>28571</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="34">
@@ -1435,10 +1435,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>20562</v>
+        <v>20000</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20562</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="35">
@@ -1463,10 +1463,10 @@
         <v>1</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>20952</v>
+        <v>20000</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20952</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="36">
@@ -1495,10 +1495,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="37">
@@ -1523,10 +1523,10 @@
         <v>1</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>19048</v>
+        <v>20000</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19048</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="38">
@@ -1551,10 +1551,10 @@
         <v>1</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>5714</v>
+        <v>5000</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>5714</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="39">
@@ -1583,10 +1583,10 @@
         <v>1</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>4762</v>
+        <v>5000</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>4762</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="40">
@@ -1615,10 +1615,10 @@
         <v>1</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>15143</v>
+        <v>15000</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>15143</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="41">
@@ -1643,10 +1643,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>19048</v>
+        <v>17000</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>19048</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="42">
@@ -1662,7 +1662,7 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="5" t="n"/>
       <c r="H42" s="9" t="n">
-        <v>232991</v>
+        <v>237000</v>
       </c>
     </row>
     <row r="43">
@@ -1678,7 +1678,7 @@
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="5" t="n"/>
       <c r="H43" s="9" t="n">
-        <v>857143</v>
+        <v>857000</v>
       </c>
     </row>
     <row r="44">
@@ -1694,7 +1694,7 @@
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="5" t="n"/>
       <c r="H44" s="11" t="n">
-        <v>42857</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
Restore KP admin rates 7800 and tech-admin 14400
Keep venue at 348k and gross 900k with 5% VAT by adjusting the media guest line.

Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -835,10 +835,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>7000</v>
+        <v>7800</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>28000</v>
+        <v>31200</v>
       </c>
     </row>
     <row r="12">
@@ -867,10 +867,10 @@
         <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>12000</v>
+        <v>14400</v>
       </c>
     </row>
     <row r="13">
@@ -886,7 +886,7 @@
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="9" t="n">
-        <v>40000</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="14">
@@ -1643,10 +1643,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>17000</v>
+        <v>11400</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>17000</v>
+        <v>11400</v>
       </c>
     </row>
     <row r="42">
@@ -1662,7 +1662,7 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="5" t="n"/>
       <c r="H42" s="9" t="n">
-        <v>237000</v>
+        <v>231400</v>
       </c>
     </row>
     <row r="43">
@@ -1717,8 +1717,8 @@
   <mergeCells count="16">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A29:H29"/>

</xml_diff>

<commit_message>
Keep all KP rates; rebalance only event organization block
Restore broadcast staff, light, PCs, TVs and management from KP.
Adjust section 6 only; host stays at 20k; total with VAT remains 900k.

Co-authored-by: harakirijkee <harakirijkee@gmail.com>
</commit_message>
<xml_diff>
--- a/MLBB_CyberSaturday_CNY_Smeta.xlsx
+++ b/MLBB_CyberSaturday_CNY_Smeta.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смета" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Смета'!$1:$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -52,7 +54,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -76,16 +78,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -107,77 +104,33 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00B0B0B0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B0B0B0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00B0B0B0"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -617,10 +570,10 @@
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
-      <c r="H3" s="5" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -633,15 +586,15 @@
           <t>Выделение и оформление зоны под программу дня</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="6" t="n">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="7" t="n">
@@ -652,7 +605,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -665,15 +618,15 @@
           <t>Монтаж зоны до открытия, подготовка рабочих мест</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="6" t="n">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="7" t="n">
@@ -684,7 +637,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -697,15 +650,15 @@
           <t>Базовый свет, звук и видео инфраструктуры арены</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="6" t="n">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -716,7 +669,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -729,15 +682,15 @@
           <t>Интернет, экраны арены, коммутация сигналов</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="7" t="n">
@@ -748,7 +701,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -761,15 +714,15 @@
           <t>Работа площадки до 18:00</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="6" t="n">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -785,12 +738,12 @@
           <t>Итого: 1. Обеспечение площадки</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="5" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
       <c r="H9" s="9" t="n">
         <v>348000</v>
       </c>
@@ -807,10 +760,10 @@
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="H10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -823,15 +776,15 @@
           <t>Операционное решение административных вопросов на площадке</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="7" t="n">
@@ -842,7 +795,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -855,15 +808,15 @@
           <t>Техническое обеспечение: звук, экран, интернет, коммутация</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6" t="n">
+      <c r="E12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
@@ -879,12 +832,12 @@
           <t>Итого: 2. Техническое обслуживание зон</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="5" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
       <c r="H13" s="9" t="n">
         <v>45600</v>
       </c>
@@ -901,10 +854,10 @@
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="H14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -917,26 +870,26 @@
           <t>Управление эфиром, переключение камер и графики</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6" t="n">
+      <c r="E15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>22000</v>
+        <v>25000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>22000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -949,118 +902,118 @@
           <t>Внутриигровая режиссура</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6" t="n">
+      <c r="E16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Инженер по звуку</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Звук на площадке и в трансляции</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>18000</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="H17" s="7" t="n">
         <v>18000</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Инженер по звуку</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Звук на площадке и в трансляции</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Инженер трансляции</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Маршрутизация сигнала, стабильность эфира</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>15000</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Инженер трансляции</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Маршрутизация сигнала, стабильность эфира</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Режиссёр по графике</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Вывод графики в видеопоток</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>чел.</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Режиссёр по графике</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Вывод графики в видеопоток</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>чел.</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="6" t="n">
+      <c r="E19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>18000</v>
+        <v>20000</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>18000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="20">
@@ -1069,14 +1022,14 @@
           <t>Итого: 3. Медиа / трансляция</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="5" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
       <c r="H20" s="9" t="n">
-        <v>95000</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="21">
@@ -1091,10 +1044,10 @@
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
-      <c r="H21" s="5" t="n"/>
+      <c r="H21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1107,26 +1060,26 @@
           <t>Комплект студийного света</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>комплект</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="6" t="n">
+      <c r="E22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -1139,26 +1092,26 @@
           <t>Зона Genshin Impact, мини-игры; смена до 12 ч</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F23" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>9000</v>
+        <v>10440</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>36000</v>
+        <v>41760</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1171,15 +1124,15 @@
           <t>Зона Genshin Impact и показ на зоне; смена до 12 ч</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E24" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F24" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="7" t="n">
@@ -1195,14 +1148,14 @@
           <t>Итого: 4. Оборудование</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="5" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
       <c r="H25" s="9" t="n">
-        <v>67000</v>
+        <v>73760</v>
       </c>
     </row>
     <row r="26">
@@ -1217,10 +1170,10 @@
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
-      <c r="H26" s="5" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -1233,22 +1186,22 @@
           <t>Координация зоны и программы</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="6" t="n">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>70000</v>
+        <v>80000</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>70000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="28">
@@ -1257,14 +1210,14 @@
           <t>Итого: 5. Менеджмент</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="5" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
       <c r="H28" s="9" t="n">
-        <v>70000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="29">
@@ -1279,10 +1232,10 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
-      <c r="H29" s="5" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -1295,26 +1248,26 @@
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="6" t="n">
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -1327,122 +1280,122 @@
           <t>Фото весь день</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G31" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Фотозона Mobile Legends 3×2 м</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Каркас, печать, монтаж</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Декор зоны Genshin Impact</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Панели, ткань, фонари, фотофон</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="H31" s="7" t="n">
+      <c r="H33" s="7" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Фотозона Mobile Legends 3×2 м</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Каркас, печать, монтаж</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="7" t="n">
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Декор под Китайский Новый год</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Зона Mobile Legends и проходы</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H32" s="7" t="n">
+      <c r="H34" s="7" t="n">
         <v>15000</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Декор зоны Genshin Impact</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Панели, ткань, фонари, фотофон</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H33" s="7" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Декор под Китайский Новый год</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>Зона Mobile Legends и проходы</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H34" s="7" t="n">
-        <v>20000</v>
-      </c>
-    </row>
     <row r="35">
-      <c r="A35" s="6" t="n">
+      <c r="A35" s="5" t="n">
         <v>6</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1451,15 +1404,15 @@
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="6" t="n">
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G35" s="7" t="n">
@@ -1470,7 +1423,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n">
+      <c r="A36" s="5" t="n">
         <v>7</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1483,26 +1436,26 @@
           <t>Призы</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="6" t="n">
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>25000</v>
+        <v>22000</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>25000</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n">
+      <c r="A37" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1511,15 +1464,15 @@
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr"/>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G37" s="7" t="n">
@@ -1530,7 +1483,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
+      <c r="A38" s="5" t="n">
         <v>9</v>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -1539,26 +1492,26 @@
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr"/>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="6" t="n">
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="5" t="n">
         <v>10</v>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1571,26 +1524,26 @@
           <t>Валюта и оформление</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="6" t="n">
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n">
+      <c r="A40" s="5" t="n">
         <v>11</v>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -1603,26 +1556,26 @@
           <t>2 суток, с резервом</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="6" t="n">
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="5" t="n">
         <v>12</v>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -1631,22 +1584,22 @@
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr"/>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>проект</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="6" t="n">
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>11400</v>
+        <v>17640</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>11400</v>
+        <v>17640</v>
       </c>
     </row>
     <row r="42">
@@ -1655,14 +1608,14 @@
           <t>Итого: 6. Организация ивента</t>
         </is>
       </c>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="5" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
       <c r="H42" s="9" t="n">
-        <v>231400</v>
+        <v>201640</v>
       </c>
     </row>
     <row r="43">
@@ -1671,45 +1624,45 @@
           <t>Итого без НДС</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="5" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
       <c r="H43" s="9" t="n">
         <v>857000</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>НДС 5%</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="11" t="n">
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="9" t="n">
         <v>43000</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>ИТОГО с НДС</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="13" t="n">
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="10" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="10" t="n"/>
+      <c r="H45" s="11" t="n">
         <v>900000</v>
       </c>
     </row>
@@ -1717,8 +1670,8 @@
   <mergeCells count="16">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A44:G44"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A29:H29"/>

</xml_diff>